<commit_message>
municipality shapefile and clean name formatting key
</commit_message>
<xml_diff>
--- a/Necessary_Files/muni_shortnames.xlsx
+++ b/Necessary_Files/muni_shortnames.xlsx
@@ -1,27 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aleaw\OneDrive\Documents\PhD Fall 2021 - Spring 2022\Merriman RA\Levy Elasticity Research\Levy_Elasticity\Necessary_Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A803ACBA-6689-4653-AD4F-D288EF6EEA30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B366619A-3D8E-4D64-9971-C7CC3B456B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{E04B2839-4174-4D46-99FA-03AE29BCB57B}"/>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{F68F1FC2-8711-44FC-A2DE-CC6924FC6194}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="township_shapefile_variables" sheetId="3" r:id="rId3"/>
+    <sheet name="township_shapefile_variables" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId4"/>
-  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1230" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1165" uniqueCount="587">
   <si>
     <t>VILLAGE OF ALSIP</t>
   </si>
@@ -1346,12 +1341,6 @@
     <t>Most recent reassessed</t>
   </si>
   <si>
-    <t>Row Labels</t>
-  </si>
-  <si>
-    <t>Average of Most recent reassessed</t>
-  </si>
-  <si>
     <t>township_code</t>
   </si>
   <si>
@@ -1806,6 +1795,9 @@
   </si>
   <si>
     <t>clean_name_alt</t>
+  </si>
+  <si>
+    <t>McCook</t>
   </si>
 </sst>
 </file>
@@ -1903,7 +1895,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1912,10 +1904,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2121,2833 +2109,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Alea Wilbur" refreshedDate="45183.474098726852" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="134" xr:uid="{96453F7C-CC08-4E98-8CEC-506741AA0D86}">
-  <cacheSource type="worksheet">
-    <worksheetSource name="Table1"/>
-  </cacheSource>
-  <cacheFields count="9">
-    <cacheField name="agency_number" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="20060000" maxValue="31350000"/>
-    </cacheField>
-    <cacheField name="agency_name" numFmtId="0">
-      <sharedItems count="134">
-        <s v="CITY OF CHICAGO"/>
-        <s v="VILLAGE OF BARRINGTON"/>
-        <s v="VILLAGE OF BARRINGTON HILLS"/>
-        <s v="VILLAGE OF EAST DUNDEE"/>
-        <s v="VILLAGE OF SOUTH BARRINGTON"/>
-        <s v="VILLAGE OF ELK GROVE VILLAGE"/>
-        <s v="VILLAGE OF MT PROSPECT"/>
-        <s v="CITY OF EVANSTON"/>
-        <s v="CITY OF NORTH LAKE"/>
-        <s v="VILLAGE OF BENSENVILLE"/>
-        <s v="VILLAGE OF ELMWOOD PARK"/>
-        <s v="VILLAGE OF FRANKLIN PARK"/>
-        <s v="VILLAGE OF RIVER GROVE"/>
-        <s v="VILLAGE OF SCHILLER PARK"/>
-        <s v="CITY OF DES PLAINES"/>
-        <s v="CITY OF PARK RIDGE"/>
-        <s v="VILLAGE OF ROSEMONT"/>
-        <s v="VILLAGE OF GLENCOE"/>
-        <s v="VILLAGE OF KENILWORTH"/>
-        <s v="VILLAGE OF WILMETTE"/>
-        <s v="VILLAGE OF WINNETKA"/>
-        <s v="VILLAGE OF GOLF"/>
-        <s v="VILLAGE OF LINCOLNWOOD"/>
-        <s v="VILLAGE OF MORTON GROVE"/>
-        <s v="VILLAGE OF NILES"/>
-        <s v="VILLAGE OF SKOKIE"/>
-        <s v="VILLAGE OF DEERFIELD"/>
-        <s v="VILLAGE OF GLENVIEW"/>
-        <s v="VILLAGE OF NORTHBROOK"/>
-        <s v="VILLAGE OF NORTHFIELD"/>
-        <s v="VILLAGE OF OAK BROOK"/>
-        <s v="VILLAGE OF HARWOOD HEIGHTS"/>
-        <s v="VILLAGE OF NORRIDGE"/>
-        <s v="CITY OF ROLLING MEADOWS"/>
-        <s v="VILLAGE OF DEER PARK"/>
-        <s v="VILLAGE OF INVERNESS"/>
-        <s v="VILLAGE OF PALATINE"/>
-        <s v="VILLAGE OF HOFFMAN ESTATES"/>
-        <s v="VILLAGE OF ROSELLE"/>
-        <s v="VILLAGE OF SCHAUMBURG"/>
-        <s v="CITY OF PROSPECT HEIGHTS"/>
-        <s v="VILLAGE OF ARLINGTON HEIGHTS"/>
-        <s v="VILLAGE OF BUFFALO GROVE"/>
-        <s v="VILLAGE OF WHEELING"/>
-        <s v="CITY OF BERWYN"/>
-        <s v="CITY OF CHICAGO HEIGHTS"/>
-        <s v="VILLAGE OF FORD HEIGHTS"/>
-        <s v="VILLAGE OF GLENWOOD"/>
-        <s v="VILLAGE OF LYNWOOD"/>
-        <s v="VILLAGE OF SAUK VILLAGE"/>
-        <s v="VILLAGE OF SOUTH CHICAGO HEIGHTS"/>
-        <s v="VILLAGE OF STEGER"/>
-        <s v="CITY OF COUNTRY CLUB HILLS"/>
-        <s v="CITY OF MARKHAM"/>
-        <s v="CITY OF OAK FOREST"/>
-        <s v="VILLAGE OF CRESTWOOD"/>
-        <s v="VILLAGE OF HAZELCREST"/>
-        <s v="VILLAGE OF MIDLOTHIAN"/>
-        <s v="VILLAGE OF POSEN"/>
-        <s v="VILLAGE OF ROBBINS"/>
-        <s v="VILLAGE OF TINLEY PARK"/>
-        <s v="CITY OF BLUE ISLAND"/>
-        <s v="VILLAGE OF CALUMET PARK"/>
-        <s v="TOWN CICERO"/>
-        <s v="CITY OF ELGIN"/>
-        <s v="VILLAGE OF BARTLETT"/>
-        <s v="VILLAGE OF STREAMWOOD"/>
-        <s v="VILLAGE OF LEMONT"/>
-        <s v="CITY OF COUNTRYSIDE"/>
-        <s v="VILLAGE OF BRIDGEVIEW"/>
-        <s v="VILLAGE OF BURR RIDGE"/>
-        <s v="VILLAGE OF HANOVER PARK"/>
-        <s v="VILLAGE OF HINSDALE"/>
-        <s v="VILLAGE OF HODGKINS"/>
-        <s v="VILLAGE OF HOMER GLEN"/>
-        <s v="VILLAGE OF INDIAN HEAD PARK"/>
-        <s v="VILLAGE OF JUSTICE"/>
-        <s v="VILLAGE OF LA GRANGE"/>
-        <s v="VILLAGE OF LA GRANGE PARK"/>
-        <s v="VILLAGE OF LYONS"/>
-        <s v="VILLAGE OF MC COOK"/>
-        <s v="VILLAGE OF SUMMIT"/>
-        <s v="VILLAGE OF WESTERN SPRINGS"/>
-        <s v="VILLAGE OF WILLOW SPRINGS"/>
-        <s v="VILLAGE OF OAK PARK"/>
-        <s v="VILLAGE OF ORLAND HILLS"/>
-        <s v="VILLAGE OF ORLAND PARK"/>
-        <s v="CITY OF HICKORY HILLS"/>
-        <s v="CITY OF PALOS HEIGHTS"/>
-        <s v="CITY OF PALOS HILLS"/>
-        <s v="VILLAGE OF PALOS PARK"/>
-        <s v="VILLAGE OF BELLWOOD"/>
-        <s v="VILLAGE OF BERKELEY"/>
-        <s v="VILLAGE OF BROADVIEW"/>
-        <s v="VILLAGE OF BROOKFIELD"/>
-        <s v="VILLAGE OF FOREST PARK"/>
-        <s v="VILLAGE OF HILLSIDE"/>
-        <s v="VILLAGE OF MAYWOOD"/>
-        <s v="VILLAGE OF MELROSE PARK"/>
-        <s v="VILLAGE OF STONE PARK"/>
-        <s v="VILLAGE OF WESTCHESTER"/>
-        <s v="VILLAGE OF FLOSSMOOR"/>
-        <s v="VILLAGE OF FRANKFORT"/>
-        <s v="VILLAGE OF MATTESON"/>
-        <s v="VILLAGE OF OLYMPIA FIELDS"/>
-        <s v="VILLAGE OF PARK FOREST"/>
-        <s v="VILLAGE OF RICHTON PARK"/>
-        <s v="VILLAGE OF UNIVERSITY PARK"/>
-        <s v="VILLAGE OF RIVER FOREST"/>
-        <s v="VILLAGE OF NORTH RIVERSIDE"/>
-        <s v="VILLAGE OF RIVERSIDE"/>
-        <s v="CITY OF BURBANK"/>
-        <s v="VILLAGE OF BEDFORD PARK"/>
-        <s v="VILLAGE OF FORESTVIEW"/>
-        <s v="VILLAGE OF STICKNEY"/>
-        <s v="CITY OF CALUMET CITY"/>
-        <s v="CITY OF HARVEY"/>
-        <s v="VILLAGE OF BURNHAM"/>
-        <s v="VILLAGE OF DIXMOOR"/>
-        <s v="VILLAGE OF DOLTON"/>
-        <s v="VILLAGE OF EAST HAZELCREST"/>
-        <s v="VILLAGE OF HOMEWOOD"/>
-        <s v="VILLAGE OF LANSING"/>
-        <s v="VILLAGE OF PHOENIX"/>
-        <s v="VILLAGE OF RIVERDALE"/>
-        <s v="VILLAGE OF SOUTH HOLLAND"/>
-        <s v="VILLAGE OF THORNTON"/>
-        <s v="CITY OF HOMETOWN"/>
-        <s v="VILLAGE OF ALSIP"/>
-        <s v="VILLAGE OF CHICAGO RIDGE"/>
-        <s v="VILLAGE OF EVERGREEN PARK"/>
-        <s v="VILLAGE OF MERRIONETTE PARK"/>
-        <s v="VILLAGE OF OAK LAWN"/>
-        <s v="VILLAGE OF WORTH"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="short_name" numFmtId="0">
-      <sharedItems count="133">
-        <s v="CHICAGO"/>
-        <s v="BARRINGTON"/>
-        <s v="BARRINGTON HILLS"/>
-        <s v="EAST DUNDEE"/>
-        <s v="SOUTH BARRINGTON"/>
-        <s v="ELK GROVE VILLAGE"/>
-        <s v="MT PROSPECT"/>
-        <s v="EVANSTON"/>
-        <s v="NORTH LAKE"/>
-        <s v="BENSENVILLE"/>
-        <s v="ELMWOOD PARK"/>
-        <s v="FRANKLIN PARK"/>
-        <s v="RIVER GROVE"/>
-        <s v="SCHILLER PARK"/>
-        <s v="DES PLAINES"/>
-        <s v="PARK RIDGE"/>
-        <s v="ROSEMONT"/>
-        <s v="GLENCOE"/>
-        <s v="KENILWORTH"/>
-        <s v="WILMETTE"/>
-        <s v="WINNETKA"/>
-        <s v="GOLF"/>
-        <s v="LINCOLNWOOD"/>
-        <s v="MORTON GROVE"/>
-        <s v="NILES"/>
-        <s v="SKOKIE"/>
-        <s v="DEERFIELD"/>
-        <s v="GLENVIEW"/>
-        <s v="NORTHBROOK"/>
-        <s v="NORTHFIELD"/>
-        <s v="OAK BROOK"/>
-        <s v="HARWOOD HEIGHTS"/>
-        <s v="NORRIDGE"/>
-        <s v="ROLLING MEADOWS"/>
-        <s v="DEER PARK"/>
-        <s v="INVERNESS"/>
-        <s v="PALATINE"/>
-        <s v="HOFFMAN ESTATES"/>
-        <s v="ROSELLE"/>
-        <s v="SCHAUMBURG"/>
-        <s v="PROSPECT HEIGHTS"/>
-        <s v="ARLINGTON HEIGHTS"/>
-        <s v="BUFFALO GROVE"/>
-        <s v="WHEELING"/>
-        <s v="BERWYN"/>
-        <s v="CHICAGO HEIGHTS"/>
-        <s v="FORD HEIGHTS"/>
-        <s v="GLENWOOD"/>
-        <s v="LYNWOOD"/>
-        <s v="SAUK VILLAGE"/>
-        <s v="SOUTH CHICAGO HEIGHTS"/>
-        <s v="STEGER"/>
-        <s v="COUNTRY CLUB HILLS"/>
-        <s v="MARKHAM"/>
-        <s v="OAK FOREST"/>
-        <s v="CRESTWOOD"/>
-        <s v="HAZELCREST"/>
-        <s v="MIDLOTHIAN"/>
-        <s v="POSEN"/>
-        <s v="ROBBINS"/>
-        <s v="TINLEY PARK"/>
-        <s v="BLUE ISLAND"/>
-        <s v="CALUMET PARK"/>
-        <s v="CICERO"/>
-        <s v="ELGIN"/>
-        <s v="BARTLETT"/>
-        <s v="STREAMWOOD"/>
-        <s v="LEMONT"/>
-        <s v="COUNTRYSIDE"/>
-        <s v="BRIDGEVIEW"/>
-        <s v="BURR RIDGE"/>
-        <s v="HANOVER PARK"/>
-        <s v="HINSDALE"/>
-        <s v="HODGKINS"/>
-        <s v="HOMER GLEN"/>
-        <s v="INDIAN HEAD PARK"/>
-        <s v="JUSTICE"/>
-        <s v="LA GRANGE"/>
-        <s v="LA GRANGE PARK"/>
-        <s v="LYONS"/>
-        <s v="MC COOK"/>
-        <s v="SUMMIT"/>
-        <s v="WESTERN SPRINGS"/>
-        <s v="WILLOW SPRINGS"/>
-        <s v="OAK PARK"/>
-        <s v="ORLAND HILLS"/>
-        <s v="ORLAND PARK"/>
-        <s v="HICKORY HILLS"/>
-        <s v="PALOS HEIGHTS"/>
-        <s v="PALOS HILLS"/>
-        <s v="PALOS PARK"/>
-        <s v="BELLWOOD"/>
-        <s v="BERKELEY"/>
-        <s v="BROADVIEW"/>
-        <s v="BROOKFIELD"/>
-        <s v="FOREST PARK"/>
-        <s v="HILLSIDE"/>
-        <s v="MAYWOOD"/>
-        <s v="MELROSE PARK"/>
-        <s v="STONE PARK"/>
-        <s v="WESTCHESTER"/>
-        <s v="FLOSSMOOR"/>
-        <s v="FRANKFORT"/>
-        <s v="MATTESON"/>
-        <s v="OLYMPIA FIELDS"/>
-        <s v="PARK FOREST"/>
-        <s v="RICHTON PARK"/>
-        <s v="UNIVERSITY PARK"/>
-        <s v="RIVER FOREST"/>
-        <s v="NORTH RIVERSIDE"/>
-        <s v="RIVERSIDE"/>
-        <s v="BURBANK"/>
-        <s v="BEDFORD PARK"/>
-        <s v="FORESTVIEW"/>
-        <s v="STICKNEY"/>
-        <s v="CALUMET CITY"/>
-        <s v="HARVEY"/>
-        <s v="BURNHAM"/>
-        <s v="DIXMOOR"/>
-        <s v="DOLTON"/>
-        <s v="EAST HAZELCREST"/>
-        <s v="HOMEWOOD"/>
-        <s v="LANSING"/>
-        <s v="PHOENIX"/>
-        <s v="RIVERDALE"/>
-        <s v="SOUTH HOLLAND"/>
-        <s v="THORNTON"/>
-        <s v="HOMETOWN"/>
-        <s v="ALSIP"/>
-        <s v="CHICAGO RIDGE"/>
-        <s v="EVERGREEN PARK"/>
-        <s v="MERRIONETTE PARK"/>
-        <s v="OAK LAWN"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="clean_name" numFmtId="0">
-      <sharedItems count="134">
-        <s v="Chicago"/>
-        <s v="Barrington"/>
-        <s v="Barrington Hills"/>
-        <s v="East Dundee"/>
-        <s v="South Barrington"/>
-        <s v="Elk Grove Village"/>
-        <s v="Mt Prospect"/>
-        <s v="Evanston"/>
-        <s v="North Lake"/>
-        <s v="Bensenville"/>
-        <s v="Elmwood Park"/>
-        <s v="Franklin Park"/>
-        <s v="River Grove"/>
-        <s v="Schiller Park"/>
-        <s v="Des Plaines"/>
-        <s v="Park Ridge"/>
-        <s v="Rosemont"/>
-        <s v="Glencoe"/>
-        <s v="Kenilworth"/>
-        <s v="Wilmette"/>
-        <s v="Winnetka"/>
-        <s v="Golf"/>
-        <s v="Lincolnwood"/>
-        <s v="Morton Grove"/>
-        <s v="Niles"/>
-        <s v="Skokie"/>
-        <s v="Deerfield"/>
-        <s v="Glenview"/>
-        <s v="Northbrook"/>
-        <s v="Northfield"/>
-        <s v="Oak Brook"/>
-        <s v="Harwood Heights"/>
-        <s v="Norridge"/>
-        <s v="Rolling Meadows"/>
-        <s v="Deer Park"/>
-        <s v="Inverness"/>
-        <s v="Palatine"/>
-        <s v="Hoffman Estates"/>
-        <s v="Roselle"/>
-        <s v="Schaumburg"/>
-        <s v="Prospect Heights"/>
-        <s v="Arlington Heights"/>
-        <s v="Buffalo Grove"/>
-        <s v="Wheeling"/>
-        <s v="Berwyn"/>
-        <s v="Chicago Heights"/>
-        <s v="Ford Heights"/>
-        <s v="Glenwood"/>
-        <s v="Lynwood"/>
-        <s v="Sauk Village"/>
-        <s v="South Chicago Heights"/>
-        <s v="Steger"/>
-        <s v="Country Club Hills"/>
-        <s v="Markham"/>
-        <s v="Oak Forest"/>
-        <s v="Crestwood"/>
-        <s v="Hazelcrest"/>
-        <s v="Midlothian"/>
-        <s v="Posen"/>
-        <s v="Robbins"/>
-        <s v="Tinley Park"/>
-        <s v="Blue Island"/>
-        <s v="Calumet Park"/>
-        <s v="Cicero"/>
-        <s v="Elgin"/>
-        <s v="Bartlett"/>
-        <s v="Streamwood"/>
-        <s v="Lemont"/>
-        <s v="Countryside"/>
-        <s v="Bridgeview"/>
-        <s v="Burr Ridge"/>
-        <s v="Hanover Park"/>
-        <s v="Hinsdale"/>
-        <s v="Hodgkins"/>
-        <s v="Homer Glen"/>
-        <s v="Indian Head Park"/>
-        <s v="Justice"/>
-        <s v="La Grange"/>
-        <s v="La Grange Park"/>
-        <s v="Lyons"/>
-        <s v="Mc Cook"/>
-        <s v="Summit"/>
-        <s v="Western Springs"/>
-        <s v="Willow Springs"/>
-        <s v="Oak Park"/>
-        <s v="Orland Hills"/>
-        <s v="Orland Park"/>
-        <s v="Hickory Hills"/>
-        <s v="Palos Heights"/>
-        <s v="Palos Hills"/>
-        <s v="Palos Park"/>
-        <s v="Bellwood"/>
-        <s v="Berkeley"/>
-        <s v="Broadview"/>
-        <s v="Brookfield"/>
-        <s v="Forest Park"/>
-        <s v="Hillside"/>
-        <s v="Maywood"/>
-        <s v="Melrose Park"/>
-        <s v="Stone Park"/>
-        <s v="Westchester"/>
-        <s v="Flossmoor"/>
-        <s v="Frankfort"/>
-        <s v="Matteson"/>
-        <s v="Olympia Fields"/>
-        <s v="Park Forest"/>
-        <s v="Richton Park"/>
-        <s v="University Park"/>
-        <s v="River Forest"/>
-        <s v="North Riverside"/>
-        <s v="Riverside"/>
-        <s v="Burbank"/>
-        <s v="Bedford Park"/>
-        <s v="Forestview"/>
-        <s v="Stickney"/>
-        <s v="Calumet City"/>
-        <s v="Harvey"/>
-        <s v="Burnham"/>
-        <s v="Dixmoor"/>
-        <s v="Dolton"/>
-        <s v="East Hazelcrest"/>
-        <s v="Homewood"/>
-        <s v="Lansing"/>
-        <s v="Phoenix"/>
-        <s v="Riverdale"/>
-        <s v="South Holland"/>
-        <s v="Thornton"/>
-        <s v="Hometown"/>
-        <s v="Alsip"/>
-        <s v="Chicago Ridge"/>
-        <s v="Evergreen Park"/>
-        <s v="Merrionette Park"/>
-        <s v="Oak Lawn"/>
-        <s v="Worth"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="shpfile_name" numFmtId="0">
-      <sharedItems count="134">
-        <s v="Chicago"/>
-        <s v="Barrington"/>
-        <s v="Barrington Hills"/>
-        <s v="East Dundee"/>
-        <s v="South Barrington"/>
-        <s v="Elk Grove Village"/>
-        <s v="Mount Prospect"/>
-        <s v="Evanston"/>
-        <s v="Northlake"/>
-        <s v="Bensenville"/>
-        <s v="Elmwood Park"/>
-        <s v="Franklin Park"/>
-        <s v="River Grove"/>
-        <s v="Schiller Park"/>
-        <s v="Des Plaines"/>
-        <s v="Park Ridge"/>
-        <s v="Rosemont"/>
-        <s v="Glencoe"/>
-        <s v="Kenilworth"/>
-        <s v="Wilmette"/>
-        <s v="Winnetka"/>
-        <s v="Golf"/>
-        <s v="Lincolnwood"/>
-        <s v="Morton Grove"/>
-        <s v="Niles"/>
-        <s v="Skokie"/>
-        <s v="Deerfield"/>
-        <s v="Glenview"/>
-        <s v="Northbrook"/>
-        <s v="Northfield"/>
-        <s v="Oak Brook"/>
-        <s v="Harwood Heights"/>
-        <s v="Norridge"/>
-        <s v="Rolling Meadows"/>
-        <s v="Deer Park"/>
-        <s v="Inverness"/>
-        <s v="Palatine"/>
-        <s v="Hoffman Estates"/>
-        <s v="Roselle"/>
-        <s v="Schaumburg"/>
-        <s v="Prospect Heights"/>
-        <s v="Arlington Heights"/>
-        <s v="Buffalo Grove"/>
-        <s v="Wheeling"/>
-        <s v="Berwyn"/>
-        <s v="Chicago Heights"/>
-        <s v="Ford Heights"/>
-        <s v="Glenwood"/>
-        <s v="Lynwood"/>
-        <s v="Sauk Village"/>
-        <s v="South Chicago Heights"/>
-        <s v="Steger"/>
-        <s v="Country Club Hills"/>
-        <s v="Markham"/>
-        <s v="Oak Forest"/>
-        <s v="Crestwood"/>
-        <s v="Hazel Crest"/>
-        <s v="Midlothian"/>
-        <s v="Posen"/>
-        <s v="Robbins"/>
-        <s v="Tinley Park"/>
-        <s v="Blue Island"/>
-        <s v="Calumet Park"/>
-        <s v="Cicero"/>
-        <s v="Elgin"/>
-        <s v="Bartlett"/>
-        <s v="Streamwood"/>
-        <s v="Lemont"/>
-        <s v="Countryside"/>
-        <s v="Bridgeview"/>
-        <s v="Burr Ridge"/>
-        <s v="Hanover Park"/>
-        <s v="Hinsdale"/>
-        <s v="Hodgkins"/>
-        <s v="Homer Glen"/>
-        <s v="Indian Head Park"/>
-        <s v="Justice"/>
-        <s v="La Grange"/>
-        <s v="La Grange Park"/>
-        <s v="Lyons"/>
-        <s v="Mc Cook"/>
-        <s v="Summit"/>
-        <s v="Western Springs"/>
-        <s v="Willow Springs"/>
-        <s v="Oak Park"/>
-        <s v="Orland Hills"/>
-        <s v="Orland Park"/>
-        <s v="Hickory Hills"/>
-        <s v="Palos Heights"/>
-        <s v="Palos Hills"/>
-        <s v="Palos Park"/>
-        <s v="Bellwood"/>
-        <s v="Berkeley"/>
-        <s v="Broadview"/>
-        <s v="Brookfield"/>
-        <s v="Forest Park"/>
-        <s v="Hillside"/>
-        <s v="Maywood"/>
-        <s v="Melrose Park"/>
-        <s v="Stone Park"/>
-        <s v="Westchester"/>
-        <s v="Flossmoor"/>
-        <s v="Frankfort"/>
-        <s v="Matteson"/>
-        <s v="Olympia Fields"/>
-        <s v="Park Forest"/>
-        <s v="Richton Park"/>
-        <s v="University Park"/>
-        <s v="River Forest"/>
-        <s v="North Riverside"/>
-        <s v="Riverside"/>
-        <s v="Burbank"/>
-        <s v="Bedford Park"/>
-        <s v="Forest View"/>
-        <s v="Stickney"/>
-        <s v="Calumet City"/>
-        <s v="Harvey"/>
-        <s v="Burnham"/>
-        <s v="Dixmoor"/>
-        <s v="Dolton"/>
-        <s v="East Hazel Crest"/>
-        <s v="Homewood"/>
-        <s v="Lansing"/>
-        <s v="Phoenix"/>
-        <s v="Riverdale"/>
-        <s v="South Holland"/>
-        <s v="Thornton"/>
-        <s v="Hometown"/>
-        <s v="Alsip"/>
-        <s v="Chicago Ridge"/>
-        <s v="Evergreen Park"/>
-        <s v="Merrionette Park"/>
-        <s v="Oak Lawn"/>
-        <s v="Worth"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Triad" numFmtId="0">
-      <sharedItems count="3">
-        <s v="City"/>
-        <s v="North"/>
-        <s v="South"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Township" numFmtId="0">
-      <sharedItems count="31">
-        <s v="Chicago"/>
-        <s v="Barrington"/>
-        <s v="Elk Grove"/>
-        <s v="Evanston"/>
-        <s v="Leyden"/>
-        <s v="Maine"/>
-        <s v="New Trier"/>
-        <s v="Niles"/>
-        <s v="Northfield"/>
-        <s v="Norwood Park"/>
-        <s v="Palatine"/>
-        <s v="Schaumburg"/>
-        <s v="Wheeling"/>
-        <s v="Berwyn"/>
-        <s v="Bloom"/>
-        <s v="Bremen"/>
-        <s v="Calumet"/>
-        <s v="Cicero"/>
-        <s v="Hanover"/>
-        <s v="Lemont"/>
-        <s v="Lyons"/>
-        <s v="Oak Park"/>
-        <s v="Orland"/>
-        <s v="Palos"/>
-        <s v="Proviso"/>
-        <s v="Rich"/>
-        <s v="River Forest"/>
-        <s v="Riverside"/>
-        <s v="Stickney"/>
-        <s v="Thornton"/>
-        <s v="Worth"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Column1" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Most recent reassessed" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="2019" maxValue="2021"/>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="134">
-  <r>
-    <n v="30210000"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-    <m/>
-    <n v="2021"/>
-  </r>
-  <r>
-    <n v="30030000"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30040000"/>
-    <x v="2"/>
-    <x v="2"/>
-    <x v="2"/>
-    <x v="2"/>
-    <x v="1"/>
-    <x v="1"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30320000"/>
-    <x v="3"/>
-    <x v="3"/>
-    <x v="3"/>
-    <x v="3"/>
-    <x v="1"/>
-    <x v="1"/>
-    <s v="OUT"/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31180000"/>
-    <x v="4"/>
-    <x v="4"/>
-    <x v="4"/>
-    <x v="4"/>
-    <x v="1"/>
-    <x v="1"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30350000"/>
-    <x v="5"/>
-    <x v="5"/>
-    <x v="5"/>
-    <x v="5"/>
-    <x v="1"/>
-    <x v="2"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30820000"/>
-    <x v="6"/>
-    <x v="6"/>
-    <x v="6"/>
-    <x v="6"/>
-    <x v="1"/>
-    <x v="2"/>
-    <s v="Wheeling"/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30380000"/>
-    <x v="7"/>
-    <x v="7"/>
-    <x v="7"/>
-    <x v="7"/>
-    <x v="1"/>
-    <x v="3"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30850000"/>
-    <x v="8"/>
-    <x v="8"/>
-    <x v="8"/>
-    <x v="8"/>
-    <x v="1"/>
-    <x v="4"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30080000"/>
-    <x v="9"/>
-    <x v="9"/>
-    <x v="9"/>
-    <x v="9"/>
-    <x v="1"/>
-    <x v="4"/>
-    <s v="OUT"/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30370000"/>
-    <x v="10"/>
-    <x v="10"/>
-    <x v="10"/>
-    <x v="10"/>
-    <x v="1"/>
-    <x v="4"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30450000"/>
-    <x v="11"/>
-    <x v="11"/>
-    <x v="11"/>
-    <x v="11"/>
-    <x v="1"/>
-    <x v="4"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31070000"/>
-    <x v="12"/>
-    <x v="12"/>
-    <x v="12"/>
-    <x v="12"/>
-    <x v="1"/>
-    <x v="4"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31160000"/>
-    <x v="13"/>
-    <x v="13"/>
-    <x v="13"/>
-    <x v="13"/>
-    <x v="1"/>
-    <x v="4"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30290000"/>
-    <x v="14"/>
-    <x v="14"/>
-    <x v="14"/>
-    <x v="14"/>
-    <x v="1"/>
-    <x v="5"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31010000"/>
-    <x v="15"/>
-    <x v="15"/>
-    <x v="15"/>
-    <x v="15"/>
-    <x v="1"/>
-    <x v="5"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31130000"/>
-    <x v="16"/>
-    <x v="16"/>
-    <x v="16"/>
-    <x v="16"/>
-    <x v="1"/>
-    <x v="5"/>
-    <s v="Leydon"/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30460000"/>
-    <x v="17"/>
-    <x v="17"/>
-    <x v="17"/>
-    <x v="17"/>
-    <x v="1"/>
-    <x v="6"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30650000"/>
-    <x v="18"/>
-    <x v="18"/>
-    <x v="18"/>
-    <x v="18"/>
-    <x v="1"/>
-    <x v="6"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31330000"/>
-    <x v="19"/>
-    <x v="19"/>
-    <x v="19"/>
-    <x v="19"/>
-    <x v="1"/>
-    <x v="6"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31340000"/>
-    <x v="20"/>
-    <x v="20"/>
-    <x v="20"/>
-    <x v="20"/>
-    <x v="1"/>
-    <x v="6"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30490000"/>
-    <x v="21"/>
-    <x v="21"/>
-    <x v="21"/>
-    <x v="21"/>
-    <x v="1"/>
-    <x v="7"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30700000"/>
-    <x v="22"/>
-    <x v="22"/>
-    <x v="22"/>
-    <x v="22"/>
-    <x v="1"/>
-    <x v="7"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30810000"/>
-    <x v="23"/>
-    <x v="23"/>
-    <x v="23"/>
-    <x v="23"/>
-    <x v="1"/>
-    <x v="7"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30830000"/>
-    <x v="24"/>
-    <x v="24"/>
-    <x v="24"/>
-    <x v="24"/>
-    <x v="1"/>
-    <x v="7"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31170000"/>
-    <x v="25"/>
-    <x v="25"/>
-    <x v="25"/>
-    <x v="25"/>
-    <x v="1"/>
-    <x v="7"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30280000"/>
-    <x v="26"/>
-    <x v="26"/>
-    <x v="26"/>
-    <x v="26"/>
-    <x v="1"/>
-    <x v="8"/>
-    <s v="OUT"/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30470000"/>
-    <x v="27"/>
-    <x v="27"/>
-    <x v="27"/>
-    <x v="27"/>
-    <x v="1"/>
-    <x v="8"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30870000"/>
-    <x v="28"/>
-    <x v="28"/>
-    <x v="28"/>
-    <x v="28"/>
-    <x v="1"/>
-    <x v="8"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30880000"/>
-    <x v="29"/>
-    <x v="29"/>
-    <x v="29"/>
-    <x v="29"/>
-    <x v="1"/>
-    <x v="8"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30890000"/>
-    <x v="30"/>
-    <x v="30"/>
-    <x v="30"/>
-    <x v="30"/>
-    <x v="1"/>
-    <x v="8"/>
-    <s v="OUT"/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30520000"/>
-    <x v="31"/>
-    <x v="31"/>
-    <x v="31"/>
-    <x v="31"/>
-    <x v="1"/>
-    <x v="9"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30840000"/>
-    <x v="32"/>
-    <x v="32"/>
-    <x v="32"/>
-    <x v="32"/>
-    <x v="1"/>
-    <x v="9"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31110000"/>
-    <x v="33"/>
-    <x v="33"/>
-    <x v="33"/>
-    <x v="33"/>
-    <x v="1"/>
-    <x v="10"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30270000"/>
-    <x v="34"/>
-    <x v="34"/>
-    <x v="34"/>
-    <x v="34"/>
-    <x v="1"/>
-    <x v="10"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30630000"/>
-    <x v="35"/>
-    <x v="35"/>
-    <x v="35"/>
-    <x v="35"/>
-    <x v="1"/>
-    <x v="10"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30960000"/>
-    <x v="36"/>
-    <x v="36"/>
-    <x v="36"/>
-    <x v="36"/>
-    <x v="1"/>
-    <x v="10"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30580000"/>
-    <x v="37"/>
-    <x v="37"/>
-    <x v="37"/>
-    <x v="37"/>
-    <x v="1"/>
-    <x v="11"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31120000"/>
-    <x v="38"/>
-    <x v="38"/>
-    <x v="38"/>
-    <x v="38"/>
-    <x v="1"/>
-    <x v="11"/>
-    <s v="OUT"/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31150000"/>
-    <x v="39"/>
-    <x v="39"/>
-    <x v="39"/>
-    <x v="39"/>
-    <x v="1"/>
-    <x v="11"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31040000"/>
-    <x v="40"/>
-    <x v="40"/>
-    <x v="40"/>
-    <x v="40"/>
-    <x v="1"/>
-    <x v="12"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30020000"/>
-    <x v="41"/>
-    <x v="41"/>
-    <x v="41"/>
-    <x v="41"/>
-    <x v="1"/>
-    <x v="12"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30150000"/>
-    <x v="42"/>
-    <x v="42"/>
-    <x v="42"/>
-    <x v="42"/>
-    <x v="1"/>
-    <x v="12"/>
-    <s v="OUT"/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31310000"/>
-    <x v="43"/>
-    <x v="43"/>
-    <x v="43"/>
-    <x v="43"/>
-    <x v="1"/>
-    <x v="12"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30100000"/>
-    <x v="44"/>
-    <x v="44"/>
-    <x v="44"/>
-    <x v="44"/>
-    <x v="2"/>
-    <x v="13"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30220000"/>
-    <x v="45"/>
-    <x v="45"/>
-    <x v="45"/>
-    <x v="45"/>
-    <x v="2"/>
-    <x v="14"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30410000"/>
-    <x v="46"/>
-    <x v="46"/>
-    <x v="46"/>
-    <x v="46"/>
-    <x v="2"/>
-    <x v="14"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30480000"/>
-    <x v="47"/>
-    <x v="47"/>
-    <x v="47"/>
-    <x v="47"/>
-    <x v="2"/>
-    <x v="14"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30710000"/>
-    <x v="48"/>
-    <x v="48"/>
-    <x v="48"/>
-    <x v="48"/>
-    <x v="2"/>
-    <x v="14"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31140000"/>
-    <x v="49"/>
-    <x v="49"/>
-    <x v="49"/>
-    <x v="49"/>
-    <x v="2"/>
-    <x v="14"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31190000"/>
-    <x v="50"/>
-    <x v="50"/>
-    <x v="50"/>
-    <x v="50"/>
-    <x v="2"/>
-    <x v="14"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31210000"/>
-    <x v="51"/>
-    <x v="51"/>
-    <x v="51"/>
-    <x v="51"/>
-    <x v="2"/>
-    <x v="14"/>
-    <s v="OUT"/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30240000"/>
-    <x v="52"/>
-    <x v="52"/>
-    <x v="52"/>
-    <x v="52"/>
-    <x v="2"/>
-    <x v="15"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30730000"/>
-    <x v="53"/>
-    <x v="53"/>
-    <x v="53"/>
-    <x v="53"/>
-    <x v="2"/>
-    <x v="15"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30900000"/>
-    <x v="54"/>
-    <x v="54"/>
-    <x v="54"/>
-    <x v="54"/>
-    <x v="2"/>
-    <x v="15"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30260000"/>
-    <x v="55"/>
-    <x v="55"/>
-    <x v="55"/>
-    <x v="55"/>
-    <x v="2"/>
-    <x v="15"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30530000"/>
-    <x v="56"/>
-    <x v="56"/>
-    <x v="56"/>
-    <x v="56"/>
-    <x v="2"/>
-    <x v="15"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30800000"/>
-    <x v="57"/>
-    <x v="57"/>
-    <x v="57"/>
-    <x v="57"/>
-    <x v="2"/>
-    <x v="15"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31030000"/>
-    <x v="58"/>
-    <x v="58"/>
-    <x v="58"/>
-    <x v="58"/>
-    <x v="2"/>
-    <x v="15"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31100000"/>
-    <x v="59"/>
-    <x v="59"/>
-    <x v="59"/>
-    <x v="59"/>
-    <x v="2"/>
-    <x v="15"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31270000"/>
-    <x v="60"/>
-    <x v="60"/>
-    <x v="60"/>
-    <x v="60"/>
-    <x v="2"/>
-    <x v="15"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30110000"/>
-    <x v="61"/>
-    <x v="61"/>
-    <x v="61"/>
-    <x v="61"/>
-    <x v="2"/>
-    <x v="16"/>
-    <s v="Worth?"/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30200000"/>
-    <x v="62"/>
-    <x v="62"/>
-    <x v="62"/>
-    <x v="62"/>
-    <x v="2"/>
-    <x v="16"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="20060000"/>
-    <x v="63"/>
-    <x v="63"/>
-    <x v="63"/>
-    <x v="63"/>
-    <x v="2"/>
-    <x v="17"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30340000"/>
-    <x v="64"/>
-    <x v="64"/>
-    <x v="64"/>
-    <x v="64"/>
-    <x v="1"/>
-    <x v="18"/>
-    <s v="OUT"/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30050000"/>
-    <x v="65"/>
-    <x v="65"/>
-    <x v="65"/>
-    <x v="65"/>
-    <x v="1"/>
-    <x v="18"/>
-    <s v="OUT"/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="31240000"/>
-    <x v="66"/>
-    <x v="66"/>
-    <x v="66"/>
-    <x v="66"/>
-    <x v="1"/>
-    <x v="18"/>
-    <m/>
-    <n v="2019"/>
-  </r>
-  <r>
-    <n v="30690000"/>
-    <x v="67"/>
-    <x v="67"/>
-    <x v="67"/>
-    <x v="67"/>
-    <x v="2"/>
-    <x v="19"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30250000"/>
-    <x v="68"/>
-    <x v="68"/>
-    <x v="68"/>
-    <x v="68"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30120000"/>
-    <x v="69"/>
-    <x v="69"/>
-    <x v="69"/>
-    <x v="69"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30180000"/>
-    <x v="70"/>
-    <x v="70"/>
-    <x v="70"/>
-    <x v="70"/>
-    <x v="2"/>
-    <x v="20"/>
-    <s v="OUT"/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30500000"/>
-    <x v="71"/>
-    <x v="71"/>
-    <x v="71"/>
-    <x v="71"/>
-    <x v="2"/>
-    <x v="20"/>
-    <s v="OUT"/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30560000"/>
-    <x v="72"/>
-    <x v="72"/>
-    <x v="72"/>
-    <x v="72"/>
-    <x v="2"/>
-    <x v="20"/>
-    <s v="OUT"/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30570000"/>
-    <x v="73"/>
-    <x v="73"/>
-    <x v="73"/>
-    <x v="73"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30585000"/>
-    <x v="74"/>
-    <x v="74"/>
-    <x v="74"/>
-    <x v="74"/>
-    <x v="2"/>
-    <x v="20"/>
-    <s v="OUT"/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30610000"/>
-    <x v="75"/>
-    <x v="75"/>
-    <x v="75"/>
-    <x v="75"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30640000"/>
-    <x v="76"/>
-    <x v="76"/>
-    <x v="76"/>
-    <x v="76"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30660000"/>
-    <x v="77"/>
-    <x v="77"/>
-    <x v="77"/>
-    <x v="77"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30670000"/>
-    <x v="78"/>
-    <x v="78"/>
-    <x v="78"/>
-    <x v="78"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30720000"/>
-    <x v="79"/>
-    <x v="79"/>
-    <x v="79"/>
-    <x v="79"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30760000"/>
-    <x v="80"/>
-    <x v="80"/>
-    <x v="80"/>
-    <x v="80"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31250000"/>
-    <x v="81"/>
-    <x v="81"/>
-    <x v="81"/>
-    <x v="81"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31300000"/>
-    <x v="82"/>
-    <x v="82"/>
-    <x v="82"/>
-    <x v="82"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31320000"/>
-    <x v="83"/>
-    <x v="83"/>
-    <x v="83"/>
-    <x v="83"/>
-    <x v="2"/>
-    <x v="20"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30920000"/>
-    <x v="84"/>
-    <x v="84"/>
-    <x v="84"/>
-    <x v="84"/>
-    <x v="2"/>
-    <x v="21"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30940000"/>
-    <x v="85"/>
-    <x v="85"/>
-    <x v="85"/>
-    <x v="85"/>
-    <x v="2"/>
-    <x v="22"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30950000"/>
-    <x v="86"/>
-    <x v="86"/>
-    <x v="86"/>
-    <x v="86"/>
-    <x v="2"/>
-    <x v="22"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30540000"/>
-    <x v="87"/>
-    <x v="87"/>
-    <x v="87"/>
-    <x v="87"/>
-    <x v="2"/>
-    <x v="23"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30970000"/>
-    <x v="88"/>
-    <x v="88"/>
-    <x v="88"/>
-    <x v="88"/>
-    <x v="2"/>
-    <x v="23"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30980000"/>
-    <x v="89"/>
-    <x v="89"/>
-    <x v="89"/>
-    <x v="89"/>
-    <x v="2"/>
-    <x v="23"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30990000"/>
-    <x v="90"/>
-    <x v="90"/>
-    <x v="90"/>
-    <x v="90"/>
-    <x v="2"/>
-    <x v="23"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30070000"/>
-    <x v="91"/>
-    <x v="91"/>
-    <x v="91"/>
-    <x v="91"/>
-    <x v="2"/>
-    <x v="24"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30090000"/>
-    <x v="92"/>
-    <x v="92"/>
-    <x v="92"/>
-    <x v="92"/>
-    <x v="2"/>
-    <x v="24"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30130000"/>
-    <x v="93"/>
-    <x v="93"/>
-    <x v="93"/>
-    <x v="93"/>
-    <x v="2"/>
-    <x v="24"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30140000"/>
-    <x v="94"/>
-    <x v="94"/>
-    <x v="94"/>
-    <x v="94"/>
-    <x v="2"/>
-    <x v="24"/>
-    <s v="Riverside"/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30420000"/>
-    <x v="95"/>
-    <x v="95"/>
-    <x v="95"/>
-    <x v="95"/>
-    <x v="2"/>
-    <x v="24"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30550000"/>
-    <x v="96"/>
-    <x v="96"/>
-    <x v="96"/>
-    <x v="96"/>
-    <x v="2"/>
-    <x v="24"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30750000"/>
-    <x v="97"/>
-    <x v="97"/>
-    <x v="97"/>
-    <x v="97"/>
-    <x v="2"/>
-    <x v="24"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30770000"/>
-    <x v="98"/>
-    <x v="98"/>
-    <x v="98"/>
-    <x v="98"/>
-    <x v="2"/>
-    <x v="24"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31230000"/>
-    <x v="99"/>
-    <x v="99"/>
-    <x v="99"/>
-    <x v="99"/>
-    <x v="2"/>
-    <x v="24"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31290000"/>
-    <x v="100"/>
-    <x v="100"/>
-    <x v="100"/>
-    <x v="100"/>
-    <x v="2"/>
-    <x v="24"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30400000"/>
-    <x v="101"/>
-    <x v="101"/>
-    <x v="101"/>
-    <x v="101"/>
-    <x v="2"/>
-    <x v="25"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30440000"/>
-    <x v="102"/>
-    <x v="102"/>
-    <x v="102"/>
-    <x v="102"/>
-    <x v="2"/>
-    <x v="25"/>
-    <s v="OUT"/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30740000"/>
-    <x v="103"/>
-    <x v="103"/>
-    <x v="103"/>
-    <x v="103"/>
-    <x v="2"/>
-    <x v="25"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30930000"/>
-    <x v="104"/>
-    <x v="104"/>
-    <x v="104"/>
-    <x v="104"/>
-    <x v="2"/>
-    <x v="25"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31000000"/>
-    <x v="105"/>
-    <x v="105"/>
-    <x v="105"/>
-    <x v="105"/>
-    <x v="2"/>
-    <x v="25"/>
-    <s v="OUT"/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31050000"/>
-    <x v="106"/>
-    <x v="106"/>
-    <x v="106"/>
-    <x v="106"/>
-    <x v="2"/>
-    <x v="25"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31280000"/>
-    <x v="107"/>
-    <x v="107"/>
-    <x v="107"/>
-    <x v="107"/>
-    <x v="2"/>
-    <x v="25"/>
-    <s v="OUT"/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31060000"/>
-    <x v="108"/>
-    <x v="108"/>
-    <x v="108"/>
-    <x v="108"/>
-    <x v="2"/>
-    <x v="26"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30860000"/>
-    <x v="109"/>
-    <x v="109"/>
-    <x v="109"/>
-    <x v="109"/>
-    <x v="2"/>
-    <x v="27"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31090000"/>
-    <x v="110"/>
-    <x v="110"/>
-    <x v="110"/>
-    <x v="110"/>
-    <x v="2"/>
-    <x v="27"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30160000"/>
-    <x v="111"/>
-    <x v="111"/>
-    <x v="111"/>
-    <x v="111"/>
-    <x v="2"/>
-    <x v="28"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30060000"/>
-    <x v="112"/>
-    <x v="112"/>
-    <x v="112"/>
-    <x v="112"/>
-    <x v="2"/>
-    <x v="28"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30430000"/>
-    <x v="113"/>
-    <x v="113"/>
-    <x v="113"/>
-    <x v="113"/>
-    <x v="2"/>
-    <x v="28"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31220000"/>
-    <x v="114"/>
-    <x v="114"/>
-    <x v="114"/>
-    <x v="114"/>
-    <x v="2"/>
-    <x v="28"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30190000"/>
-    <x v="115"/>
-    <x v="115"/>
-    <x v="115"/>
-    <x v="115"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30510000"/>
-    <x v="116"/>
-    <x v="116"/>
-    <x v="116"/>
-    <x v="116"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30170000"/>
-    <x v="117"/>
-    <x v="117"/>
-    <x v="117"/>
-    <x v="117"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30300000"/>
-    <x v="118"/>
-    <x v="118"/>
-    <x v="118"/>
-    <x v="118"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30310000"/>
-    <x v="119"/>
-    <x v="119"/>
-    <x v="119"/>
-    <x v="119"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30330000"/>
-    <x v="120"/>
-    <x v="120"/>
-    <x v="120"/>
-    <x v="120"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30600000"/>
-    <x v="121"/>
-    <x v="121"/>
-    <x v="121"/>
-    <x v="121"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30680000"/>
-    <x v="122"/>
-    <x v="122"/>
-    <x v="122"/>
-    <x v="122"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31020000"/>
-    <x v="123"/>
-    <x v="123"/>
-    <x v="123"/>
-    <x v="123"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31080000"/>
-    <x v="124"/>
-    <x v="124"/>
-    <x v="124"/>
-    <x v="124"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31200000"/>
-    <x v="125"/>
-    <x v="125"/>
-    <x v="125"/>
-    <x v="125"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31260000"/>
-    <x v="126"/>
-    <x v="126"/>
-    <x v="126"/>
-    <x v="126"/>
-    <x v="2"/>
-    <x v="29"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30590000"/>
-    <x v="127"/>
-    <x v="127"/>
-    <x v="127"/>
-    <x v="127"/>
-    <x v="2"/>
-    <x v="30"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30010000"/>
-    <x v="128"/>
-    <x v="128"/>
-    <x v="128"/>
-    <x v="128"/>
-    <x v="2"/>
-    <x v="30"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30230000"/>
-    <x v="129"/>
-    <x v="129"/>
-    <x v="129"/>
-    <x v="129"/>
-    <x v="2"/>
-    <x v="30"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30390000"/>
-    <x v="130"/>
-    <x v="130"/>
-    <x v="130"/>
-    <x v="130"/>
-    <x v="2"/>
-    <x v="30"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30780000"/>
-    <x v="131"/>
-    <x v="131"/>
-    <x v="131"/>
-    <x v="131"/>
-    <x v="2"/>
-    <x v="30"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="30910000"/>
-    <x v="132"/>
-    <x v="132"/>
-    <x v="132"/>
-    <x v="132"/>
-    <x v="2"/>
-    <x v="30"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-  <r>
-    <n v="31350000"/>
-    <x v="133"/>
-    <x v="20"/>
-    <x v="133"/>
-    <x v="133"/>
-    <x v="2"/>
-    <x v="30"/>
-    <m/>
-    <n v="2020"/>
-  </r>
-</pivotCacheRecords>
-</file>
-
-<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7B87FB73-5E5B-4C64-8111-F9E15E4E82E7}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:C34" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
-  <pivotFields count="9">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="135">
-        <item x="44"/>
-        <item x="61"/>
-        <item x="111"/>
-        <item x="115"/>
-        <item x="0"/>
-        <item x="45"/>
-        <item x="52"/>
-        <item x="68"/>
-        <item x="14"/>
-        <item x="64"/>
-        <item x="7"/>
-        <item x="116"/>
-        <item x="87"/>
-        <item x="127"/>
-        <item x="53"/>
-        <item x="8"/>
-        <item x="54"/>
-        <item x="88"/>
-        <item x="89"/>
-        <item x="15"/>
-        <item x="40"/>
-        <item x="33"/>
-        <item x="63"/>
-        <item x="128"/>
-        <item x="41"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="65"/>
-        <item x="112"/>
-        <item x="91"/>
-        <item x="9"/>
-        <item x="92"/>
-        <item x="69"/>
-        <item x="93"/>
-        <item x="94"/>
-        <item x="42"/>
-        <item x="117"/>
-        <item x="70"/>
-        <item x="62"/>
-        <item x="129"/>
-        <item x="55"/>
-        <item x="34"/>
-        <item x="26"/>
-        <item x="118"/>
-        <item x="119"/>
-        <item x="3"/>
-        <item x="120"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="130"/>
-        <item x="101"/>
-        <item x="46"/>
-        <item x="95"/>
-        <item x="113"/>
-        <item x="102"/>
-        <item x="11"/>
-        <item x="17"/>
-        <item x="27"/>
-        <item x="47"/>
-        <item x="21"/>
-        <item x="71"/>
-        <item x="31"/>
-        <item x="56"/>
-        <item x="96"/>
-        <item x="72"/>
-        <item x="73"/>
-        <item x="37"/>
-        <item x="74"/>
-        <item x="121"/>
-        <item x="75"/>
-        <item x="35"/>
-        <item x="76"/>
-        <item x="18"/>
-        <item x="77"/>
-        <item x="78"/>
-        <item x="122"/>
-        <item x="67"/>
-        <item x="22"/>
-        <item x="48"/>
-        <item x="79"/>
-        <item x="103"/>
-        <item x="97"/>
-        <item x="80"/>
-        <item x="98"/>
-        <item x="131"/>
-        <item x="57"/>
-        <item x="23"/>
-        <item x="6"/>
-        <item x="24"/>
-        <item x="32"/>
-        <item x="109"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="30"/>
-        <item x="132"/>
-        <item x="84"/>
-        <item x="104"/>
-        <item x="85"/>
-        <item x="86"/>
-        <item x="36"/>
-        <item x="90"/>
-        <item x="105"/>
-        <item x="123"/>
-        <item x="58"/>
-        <item x="106"/>
-        <item x="108"/>
-        <item x="12"/>
-        <item x="124"/>
-        <item x="110"/>
-        <item x="59"/>
-        <item x="38"/>
-        <item x="16"/>
-        <item x="49"/>
-        <item x="39"/>
-        <item x="13"/>
-        <item x="25"/>
-        <item x="4"/>
-        <item x="50"/>
-        <item x="125"/>
-        <item x="51"/>
-        <item x="114"/>
-        <item x="99"/>
-        <item x="66"/>
-        <item x="81"/>
-        <item x="126"/>
-        <item x="60"/>
-        <item x="107"/>
-        <item x="100"/>
-        <item x="82"/>
-        <item x="43"/>
-        <item x="83"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="133"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="134">
-        <item x="128"/>
-        <item x="41"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="65"/>
-        <item x="112"/>
-        <item x="91"/>
-        <item x="9"/>
-        <item x="92"/>
-        <item x="44"/>
-        <item x="61"/>
-        <item x="69"/>
-        <item x="93"/>
-        <item x="94"/>
-        <item x="42"/>
-        <item x="111"/>
-        <item x="117"/>
-        <item x="70"/>
-        <item x="115"/>
-        <item x="62"/>
-        <item x="0"/>
-        <item x="45"/>
-        <item x="129"/>
-        <item x="63"/>
-        <item x="52"/>
-        <item x="68"/>
-        <item x="55"/>
-        <item x="34"/>
-        <item x="26"/>
-        <item x="14"/>
-        <item x="118"/>
-        <item x="119"/>
-        <item x="3"/>
-        <item x="120"/>
-        <item x="64"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="7"/>
-        <item x="130"/>
-        <item x="101"/>
-        <item x="46"/>
-        <item x="95"/>
-        <item x="113"/>
-        <item x="102"/>
-        <item x="11"/>
-        <item x="17"/>
-        <item x="27"/>
-        <item x="47"/>
-        <item x="21"/>
-        <item x="71"/>
-        <item x="116"/>
-        <item x="31"/>
-        <item x="56"/>
-        <item x="87"/>
-        <item x="96"/>
-        <item x="72"/>
-        <item x="73"/>
-        <item x="37"/>
-        <item x="74"/>
-        <item x="127"/>
-        <item x="121"/>
-        <item x="75"/>
-        <item x="35"/>
-        <item x="76"/>
-        <item x="18"/>
-        <item x="77"/>
-        <item x="78"/>
-        <item x="122"/>
-        <item x="67"/>
-        <item x="22"/>
-        <item x="48"/>
-        <item x="79"/>
-        <item x="53"/>
-        <item x="103"/>
-        <item x="97"/>
-        <item x="80"/>
-        <item x="98"/>
-        <item x="131"/>
-        <item x="57"/>
-        <item x="23"/>
-        <item x="6"/>
-        <item x="24"/>
-        <item x="32"/>
-        <item x="8"/>
-        <item x="109"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="30"/>
-        <item x="54"/>
-        <item x="132"/>
-        <item x="84"/>
-        <item x="104"/>
-        <item x="85"/>
-        <item x="86"/>
-        <item x="36"/>
-        <item x="88"/>
-        <item x="89"/>
-        <item x="90"/>
-        <item x="105"/>
-        <item x="15"/>
-        <item x="123"/>
-        <item x="58"/>
-        <item x="40"/>
-        <item x="106"/>
-        <item x="108"/>
-        <item x="12"/>
-        <item x="124"/>
-        <item x="110"/>
-        <item x="59"/>
-        <item x="33"/>
-        <item x="38"/>
-        <item x="16"/>
-        <item x="49"/>
-        <item x="39"/>
-        <item x="13"/>
-        <item x="25"/>
-        <item x="4"/>
-        <item x="50"/>
-        <item x="125"/>
-        <item x="51"/>
-        <item x="114"/>
-        <item x="99"/>
-        <item x="66"/>
-        <item x="81"/>
-        <item x="126"/>
-        <item x="60"/>
-        <item x="107"/>
-        <item x="100"/>
-        <item x="82"/>
-        <item x="43"/>
-        <item x="83"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="135">
-        <item x="128"/>
-        <item x="41"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="65"/>
-        <item x="112"/>
-        <item x="91"/>
-        <item x="9"/>
-        <item x="92"/>
-        <item x="44"/>
-        <item x="61"/>
-        <item x="69"/>
-        <item x="93"/>
-        <item x="94"/>
-        <item x="42"/>
-        <item x="111"/>
-        <item x="117"/>
-        <item x="70"/>
-        <item x="115"/>
-        <item x="62"/>
-        <item x="0"/>
-        <item x="45"/>
-        <item x="129"/>
-        <item x="63"/>
-        <item x="52"/>
-        <item x="68"/>
-        <item x="55"/>
-        <item x="34"/>
-        <item x="26"/>
-        <item x="14"/>
-        <item x="118"/>
-        <item x="119"/>
-        <item x="3"/>
-        <item x="120"/>
-        <item x="64"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="7"/>
-        <item x="130"/>
-        <item x="101"/>
-        <item x="46"/>
-        <item x="95"/>
-        <item x="113"/>
-        <item x="102"/>
-        <item x="11"/>
-        <item x="17"/>
-        <item x="27"/>
-        <item x="47"/>
-        <item x="21"/>
-        <item x="71"/>
-        <item x="116"/>
-        <item x="31"/>
-        <item x="56"/>
-        <item x="87"/>
-        <item x="96"/>
-        <item x="72"/>
-        <item x="73"/>
-        <item x="37"/>
-        <item x="74"/>
-        <item x="127"/>
-        <item x="121"/>
-        <item x="75"/>
-        <item x="35"/>
-        <item x="76"/>
-        <item x="18"/>
-        <item x="77"/>
-        <item x="78"/>
-        <item x="122"/>
-        <item x="67"/>
-        <item x="22"/>
-        <item x="48"/>
-        <item x="79"/>
-        <item x="53"/>
-        <item x="103"/>
-        <item x="97"/>
-        <item x="80"/>
-        <item x="98"/>
-        <item x="131"/>
-        <item x="57"/>
-        <item x="23"/>
-        <item x="6"/>
-        <item x="24"/>
-        <item x="32"/>
-        <item x="8"/>
-        <item x="109"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="30"/>
-        <item x="54"/>
-        <item x="132"/>
-        <item x="84"/>
-        <item x="104"/>
-        <item x="85"/>
-        <item x="86"/>
-        <item x="36"/>
-        <item x="88"/>
-        <item x="89"/>
-        <item x="90"/>
-        <item x="105"/>
-        <item x="15"/>
-        <item x="123"/>
-        <item x="58"/>
-        <item x="40"/>
-        <item x="106"/>
-        <item x="108"/>
-        <item x="12"/>
-        <item x="124"/>
-        <item x="110"/>
-        <item x="59"/>
-        <item x="33"/>
-        <item x="38"/>
-        <item x="16"/>
-        <item x="49"/>
-        <item x="39"/>
-        <item x="13"/>
-        <item x="25"/>
-        <item x="4"/>
-        <item x="50"/>
-        <item x="125"/>
-        <item x="51"/>
-        <item x="114"/>
-        <item x="99"/>
-        <item x="66"/>
-        <item x="81"/>
-        <item x="126"/>
-        <item x="60"/>
-        <item x="107"/>
-        <item x="100"/>
-        <item x="82"/>
-        <item x="43"/>
-        <item x="83"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="133"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="135">
-        <item x="128"/>
-        <item x="41"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="65"/>
-        <item x="112"/>
-        <item x="91"/>
-        <item x="9"/>
-        <item x="92"/>
-        <item x="44"/>
-        <item x="61"/>
-        <item x="69"/>
-        <item x="93"/>
-        <item x="94"/>
-        <item x="42"/>
-        <item x="111"/>
-        <item x="117"/>
-        <item x="70"/>
-        <item x="115"/>
-        <item x="62"/>
-        <item x="0"/>
-        <item x="45"/>
-        <item x="129"/>
-        <item x="63"/>
-        <item x="52"/>
-        <item x="68"/>
-        <item x="55"/>
-        <item x="34"/>
-        <item x="26"/>
-        <item x="14"/>
-        <item x="118"/>
-        <item x="119"/>
-        <item x="3"/>
-        <item x="120"/>
-        <item x="64"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="7"/>
-        <item x="130"/>
-        <item x="101"/>
-        <item x="46"/>
-        <item x="95"/>
-        <item x="113"/>
-        <item x="102"/>
-        <item x="11"/>
-        <item x="17"/>
-        <item x="27"/>
-        <item x="47"/>
-        <item x="21"/>
-        <item x="71"/>
-        <item x="116"/>
-        <item x="31"/>
-        <item x="56"/>
-        <item x="87"/>
-        <item x="96"/>
-        <item x="72"/>
-        <item x="73"/>
-        <item x="37"/>
-        <item x="74"/>
-        <item x="127"/>
-        <item x="121"/>
-        <item x="75"/>
-        <item x="35"/>
-        <item x="76"/>
-        <item x="18"/>
-        <item x="77"/>
-        <item x="78"/>
-        <item x="122"/>
-        <item x="67"/>
-        <item x="22"/>
-        <item x="48"/>
-        <item x="79"/>
-        <item x="53"/>
-        <item x="103"/>
-        <item x="97"/>
-        <item x="80"/>
-        <item x="98"/>
-        <item x="131"/>
-        <item x="57"/>
-        <item x="23"/>
-        <item x="6"/>
-        <item x="24"/>
-        <item x="32"/>
-        <item x="109"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="8"/>
-        <item x="30"/>
-        <item x="54"/>
-        <item x="132"/>
-        <item x="84"/>
-        <item x="104"/>
-        <item x="85"/>
-        <item x="86"/>
-        <item x="36"/>
-        <item x="88"/>
-        <item x="89"/>
-        <item x="90"/>
-        <item x="105"/>
-        <item x="15"/>
-        <item x="123"/>
-        <item x="58"/>
-        <item x="40"/>
-        <item x="106"/>
-        <item x="108"/>
-        <item x="12"/>
-        <item x="124"/>
-        <item x="110"/>
-        <item x="59"/>
-        <item x="33"/>
-        <item x="38"/>
-        <item x="16"/>
-        <item x="49"/>
-        <item x="39"/>
-        <item x="13"/>
-        <item x="25"/>
-        <item x="4"/>
-        <item x="50"/>
-        <item x="125"/>
-        <item x="51"/>
-        <item x="114"/>
-        <item x="99"/>
-        <item x="66"/>
-        <item x="81"/>
-        <item x="126"/>
-        <item x="60"/>
-        <item x="107"/>
-        <item x="100"/>
-        <item x="82"/>
-        <item x="43"/>
-        <item x="83"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="133"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-      </items>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{2946ED86-A175-432a-8AC1-64E0C546D7DE}">
-          <x14:pivotField fillDownLabels="1"/>
-        </ext>
-      </extLst>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="32">
-        <item x="1"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="0"/>
-        <item x="17"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="4"/>
-        <item x="20"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="10"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item x="27"/>
-        <item x="11"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="12"/>
-        <item x="30"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="5"/>
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="31">
-    <i>
-      <x/>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="1"/>
-      <x/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i r="1">
-      <x v="9"/>
-    </i>
-    <i r="1">
-      <x v="11"/>
-    </i>
-    <i r="1">
-      <x v="13"/>
-    </i>
-    <i r="1">
-      <x v="14"/>
-    </i>
-    <i r="1">
-      <x v="15"/>
-    </i>
-    <i r="1">
-      <x v="16"/>
-    </i>
-    <i r="1">
-      <x v="17"/>
-    </i>
-    <i r="1">
-      <x v="20"/>
-    </i>
-    <i r="1">
-      <x v="26"/>
-    </i>
-    <i r="1">
-      <x v="29"/>
-    </i>
-    <i>
-      <x v="2"/>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i r="1">
-      <x v="18"/>
-    </i>
-    <i r="1">
-      <x v="19"/>
-    </i>
-    <i r="1">
-      <x v="21"/>
-    </i>
-    <i r="1">
-      <x v="22"/>
-    </i>
-    <i r="1">
-      <x v="23"/>
-    </i>
-    <i r="1">
-      <x v="24"/>
-    </i>
-    <i r="1">
-      <x v="25"/>
-    </i>
-    <i r="1">
-      <x v="27"/>
-    </i>
-    <i r="1">
-      <x v="28"/>
-    </i>
-    <i r="1">
-      <x v="30"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average of Most recent reassessed" fld="8" subtotal="average" baseField="5" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D179A9D4-42CB-495B-8B63-9C6B4EB0A0D5}" name="Table1" displayName="Table1" ref="A1:L135" totalsRowShown="0" headerRowDxfId="12" tableBorderDxfId="11">
   <autoFilter ref="A1:L135" xr:uid="{D179A9D4-42CB-495B-8B63-9C6B4EB0A0D5}"/>
@@ -4994,9 +2155,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5034,7 +2195,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -5140,7 +2301,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5282,7 +2443,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -5318,13 +2479,13 @@
         <v>264</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>271</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>405</v>
@@ -5333,7 +2494,7 @@
         <v>406</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>422</v>
@@ -8078,7 +5239,7 @@
         <v>349</v>
       </c>
       <c r="E77" s="3" t="s">
-        <v>349</v>
+        <v>586</v>
       </c>
       <c r="F77" s="3" t="s">
         <v>349</v>
@@ -8258,7 +5419,7 @@
         <v>432</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>432</v>
+        <v>401</v>
       </c>
       <c r="F82" s="5" t="s">
         <v>401</v>
@@ -9913,37 +7074,37 @@
       </c>
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.8">
-      <c r="A128" s="12">
+      <c r="A128" s="10">
         <v>31280000</v>
       </c>
-      <c r="B128" s="12" t="s">
+      <c r="B128" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="C128" s="12" t="s">
+      <c r="C128" s="10" t="s">
         <v>249</v>
       </c>
-      <c r="D128" s="12" t="s">
+      <c r="D128" s="10" t="s">
         <v>391</v>
       </c>
-      <c r="E128" s="12" t="s">
+      <c r="E128" s="10" t="s">
         <v>391</v>
       </c>
-      <c r="F128" s="12" t="s">
+      <c r="F128" s="10" t="s">
         <v>391</v>
       </c>
-      <c r="G128" s="12">
+      <c r="G128" s="10">
         <v>42</v>
       </c>
-      <c r="H128" s="12" t="s">
-        <v>407</v>
-      </c>
-      <c r="I128" s="12" t="s">
+      <c r="H128" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="I128" s="10" t="s">
         <v>414</v>
       </c>
-      <c r="J128" s="12">
+      <c r="J128" s="10">
         <v>32</v>
       </c>
-      <c r="K128" s="13" t="s">
+      <c r="K128" s="11" t="s">
         <v>425</v>
       </c>
       <c r="L128">
@@ -9951,253 +7112,253 @@
       </c>
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.8">
-      <c r="A129" s="10">
+      <c r="A129" s="8">
         <v>31290000</v>
       </c>
-      <c r="B129" s="10" t="s">
+      <c r="B129" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="C129" s="10" t="s">
+      <c r="C129" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="D129" s="10" t="s">
+      <c r="D129" s="8" t="s">
         <v>392</v>
       </c>
-      <c r="E129" s="10" t="s">
+      <c r="E129" s="8" t="s">
         <v>392</v>
       </c>
-      <c r="F129" s="10" t="s">
+      <c r="F129" s="8" t="s">
         <v>392</v>
       </c>
-      <c r="G129" s="10">
+      <c r="G129" s="8">
         <v>3</v>
       </c>
-      <c r="H129" s="10" t="s">
-        <v>407</v>
-      </c>
-      <c r="I129" s="10" t="s">
+      <c r="H129" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="I129" s="8" t="s">
         <v>413</v>
       </c>
-      <c r="J129" s="10">
+      <c r="J129" s="8">
         <v>31</v>
       </c>
-      <c r="K129" s="11"/>
+      <c r="K129" s="9"/>
       <c r="L129">
         <v>2020</v>
       </c>
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.8">
-      <c r="A130" s="12">
+      <c r="A130" s="10">
         <v>31300000</v>
       </c>
-      <c r="B130" s="12" t="s">
+      <c r="B130" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="C130" s="12" t="s">
+      <c r="C130" s="10" t="s">
         <v>253</v>
       </c>
-      <c r="D130" s="12" t="s">
+      <c r="D130" s="10" t="s">
         <v>393</v>
       </c>
-      <c r="E130" s="12" t="s">
+      <c r="E130" s="10" t="s">
         <v>393</v>
       </c>
-      <c r="F130" s="12" t="s">
+      <c r="F130" s="10" t="s">
         <v>393</v>
       </c>
-      <c r="G130" s="12">
+      <c r="G130" s="10">
         <v>43</v>
       </c>
-      <c r="H130" s="12" t="s">
-        <v>407</v>
-      </c>
-      <c r="I130" s="12" t="s">
+      <c r="H130" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="I130" s="10" t="s">
         <v>346</v>
       </c>
-      <c r="J130" s="12">
+      <c r="J130" s="10">
         <v>21</v>
       </c>
-      <c r="K130" s="13"/>
+      <c r="K130" s="11"/>
       <c r="L130">
         <v>2020</v>
       </c>
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.8">
-      <c r="A131" s="10">
+      <c r="A131" s="8">
         <v>31310000</v>
       </c>
-      <c r="B131" s="10" t="s">
+      <c r="B131" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="C131" s="10" t="s">
+      <c r="C131" s="8" t="s">
         <v>255</v>
       </c>
-      <c r="D131" s="10" t="s">
+      <c r="D131" s="8" t="s">
         <v>394</v>
       </c>
-      <c r="E131" s="10" t="s">
+      <c r="E131" s="8" t="s">
         <v>394</v>
       </c>
-      <c r="F131" s="10" t="s">
+      <c r="F131" s="8" t="s">
         <v>394</v>
       </c>
-      <c r="G131" s="10">
+      <c r="G131" s="8">
         <v>2</v>
       </c>
-      <c r="H131" s="10" t="s">
+      <c r="H131" s="8" t="s">
         <v>410</v>
       </c>
-      <c r="I131" s="10" t="s">
+      <c r="I131" s="8" t="s">
         <v>394</v>
       </c>
-      <c r="J131" s="10">
+      <c r="J131" s="8">
         <v>38</v>
       </c>
-      <c r="K131" s="11"/>
+      <c r="K131" s="9"/>
       <c r="L131">
         <v>2019</v>
       </c>
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.8">
-      <c r="A132" s="12">
+      <c r="A132" s="10">
         <v>31320000</v>
       </c>
-      <c r="B132" s="12" t="s">
+      <c r="B132" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="C132" s="12" t="s">
+      <c r="C132" s="10" t="s">
         <v>257</v>
       </c>
-      <c r="D132" s="12" t="s">
+      <c r="D132" s="10" t="s">
         <v>395</v>
       </c>
-      <c r="E132" s="12" t="s">
+      <c r="E132" s="10" t="s">
         <v>395</v>
       </c>
-      <c r="F132" s="12" t="s">
+      <c r="F132" s="10" t="s">
         <v>395</v>
       </c>
-      <c r="G132" s="12">
+      <c r="G132" s="10">
         <v>43</v>
       </c>
-      <c r="H132" s="12" t="s">
-        <v>407</v>
-      </c>
-      <c r="I132" s="12" t="s">
+      <c r="H132" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="I132" s="10" t="s">
         <v>346</v>
       </c>
-      <c r="J132" s="12">
+      <c r="J132" s="10">
         <v>21</v>
       </c>
-      <c r="K132" s="13"/>
+      <c r="K132" s="11"/>
       <c r="L132">
         <v>2020</v>
       </c>
     </row>
     <row r="133" spans="1:12" x14ac:dyDescent="0.8">
-      <c r="A133" s="10">
+      <c r="A133" s="8">
         <v>31330000</v>
       </c>
-      <c r="B133" s="10" t="s">
+      <c r="B133" s="8" t="s">
         <v>258</v>
       </c>
-      <c r="C133" s="10" t="s">
+      <c r="C133" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="D133" s="10" t="s">
+      <c r="D133" s="8" t="s">
         <v>396</v>
       </c>
-      <c r="E133" s="10" t="s">
+      <c r="E133" s="8" t="s">
         <v>396</v>
       </c>
-      <c r="F133" s="10" t="s">
+      <c r="F133" s="8" t="s">
         <v>396</v>
       </c>
-      <c r="G133" s="10">
+      <c r="G133" s="8">
         <v>8</v>
       </c>
-      <c r="H133" s="10" t="s">
+      <c r="H133" s="8" t="s">
         <v>410</v>
       </c>
-      <c r="I133" s="10" t="s">
+      <c r="I133" s="8" t="s">
         <v>412</v>
       </c>
-      <c r="J133" s="10">
+      <c r="J133" s="8">
         <v>23</v>
       </c>
-      <c r="K133" s="11"/>
+      <c r="K133" s="9"/>
       <c r="L133">
         <v>2019</v>
       </c>
     </row>
     <row r="134" spans="1:12" x14ac:dyDescent="0.8">
-      <c r="A134" s="12">
+      <c r="A134" s="10">
         <v>31340000</v>
       </c>
-      <c r="B134" s="12" t="s">
+      <c r="B134" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="C134" s="12" t="s">
+      <c r="C134" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="D134" s="12" t="s">
+      <c r="D134" s="10" t="s">
         <v>397</v>
       </c>
-      <c r="E134" s="12" t="s">
+      <c r="E134" s="10" t="s">
         <v>397</v>
       </c>
-      <c r="F134" s="12" t="s">
+      <c r="F134" s="10" t="s">
         <v>397</v>
       </c>
-      <c r="G134" s="12">
+      <c r="G134" s="10">
         <v>8</v>
       </c>
-      <c r="H134" s="12" t="s">
+      <c r="H134" s="10" t="s">
         <v>410</v>
       </c>
-      <c r="I134" s="12" t="s">
+      <c r="I134" s="10" t="s">
         <v>412</v>
       </c>
-      <c r="J134" s="12">
+      <c r="J134" s="10">
         <v>23</v>
       </c>
-      <c r="K134" s="13"/>
+      <c r="K134" s="11"/>
       <c r="L134">
         <v>2019</v>
       </c>
     </row>
     <row r="135" spans="1:12" x14ac:dyDescent="0.8">
-      <c r="A135" s="10">
+      <c r="A135" s="8">
         <v>31350000</v>
       </c>
-      <c r="B135" s="10" t="s">
+      <c r="B135" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="C135" s="10" t="s">
+      <c r="C135" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="D135" s="10" t="s">
+      <c r="D135" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="E135" s="10" t="s">
+      <c r="E135" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="F135" s="10" t="s">
+      <c r="F135" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="G135" s="10">
+      <c r="G135" s="8">
         <v>15</v>
       </c>
-      <c r="H135" s="10" t="s">
-        <v>407</v>
-      </c>
-      <c r="I135" s="10" t="s">
+      <c r="H135" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="I135" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="J135" s="10">
+      <c r="J135" s="8">
         <v>39</v>
       </c>
-      <c r="K135" s="11"/>
+      <c r="K135" s="9"/>
       <c r="L135">
         <v>2020</v>
       </c>
@@ -10212,376 +7373,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA0CAC8E-01F2-4C07-820A-9300B90359BA}">
-  <dimension ref="A3:C34"/>
-  <sheetFormatPr defaultRowHeight="23.1" x14ac:dyDescent="0.8"/>
-  <cols>
-    <col min="1" max="1" width="12.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.46484375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.86328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.296875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A3" s="8" t="s">
-        <v>434</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>406</v>
-      </c>
-      <c r="C3" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A4" s="9" t="s">
-        <v>416</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>276</v>
-      </c>
-      <c r="C4">
-        <v>2021</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A5" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>295</v>
-      </c>
-      <c r="C5">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A6" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>424</v>
-      </c>
-      <c r="C6">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A7" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="C7">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A8" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>420</v>
-      </c>
-      <c r="C8">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A9" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>419</v>
-      </c>
-      <c r="C9">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A10" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>411</v>
-      </c>
-      <c r="C10">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A11" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>412</v>
-      </c>
-      <c r="C11">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A12" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>354</v>
-      </c>
-      <c r="C12">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A13" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>358</v>
-      </c>
-      <c r="C13">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A14" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>423</v>
-      </c>
-      <c r="C14">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A15" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>365</v>
-      </c>
-      <c r="C15">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A16" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>378</v>
-      </c>
-      <c r="C16">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A17" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>394</v>
-      </c>
-      <c r="C17">
-        <v>2019</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A18" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="C18">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A19" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>418</v>
-      </c>
-      <c r="C19">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A20" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>415</v>
-      </c>
-      <c r="C20">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A21" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>417</v>
-      </c>
-      <c r="C21">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A22" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>268</v>
-      </c>
-      <c r="C22">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A23" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>343</v>
-      </c>
-      <c r="C23">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A24" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>346</v>
-      </c>
-      <c r="C24">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A25" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>361</v>
-      </c>
-      <c r="C25">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A26" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>408</v>
-      </c>
-      <c r="C26">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A27" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>409</v>
-      </c>
-      <c r="C27">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A28" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="C28">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A29" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>414</v>
-      </c>
-      <c r="C29">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A30" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>370</v>
-      </c>
-      <c r="C30">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A31" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>373</v>
-      </c>
-      <c r="C31">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A32" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>385</v>
-      </c>
-      <c r="C32">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A33" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>389</v>
-      </c>
-      <c r="C33">
-        <v>2020</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.8">
-      <c r="A34" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>266</v>
-      </c>
-      <c r="C34">
-        <v>2020</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13708FBC-0B91-46E5-AEFC-942007A5A68A}">
   <dimension ref="A1:I40"/>
   <sheetFormatPr defaultRowHeight="23.1" x14ac:dyDescent="0.8"/>
@@ -10599,31 +7390,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.8">
       <c r="A1" t="s">
+        <v>435</v>
+      </c>
+      <c r="B1" t="s">
+        <v>436</v>
+      </c>
+      <c r="C1" t="s">
         <v>437</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>438</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>439</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>440</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>441</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>442</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>443</v>
-      </c>
-      <c r="H1" t="s">
-        <v>444</v>
-      </c>
-      <c r="I1" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.8">
@@ -10634,19 +7425,19 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D2" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="E2">
         <v>6</v>
       </c>
       <c r="F2" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="G2" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="H2">
         <v>1006173334</v>
@@ -10663,19 +7454,19 @@
         <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D3" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E3">
         <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="G3" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="H3">
         <v>108744824</v>
@@ -10689,22 +7480,22 @@
         <v>250485</v>
       </c>
       <c r="B4" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C4" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D4" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="E4">
         <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G4" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="H4">
         <v>1300305077</v>
@@ -10718,22 +7509,22 @@
         <v>250486</v>
       </c>
       <c r="B5" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="C5">
         <v>2007001374</v>
       </c>
       <c r="D5" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="E5">
         <v>41</v>
       </c>
       <c r="F5" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="G5" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="H5">
         <v>1055138598</v>
@@ -10747,22 +7538,22 @@
         <v>250487</v>
       </c>
       <c r="B6" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C6" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D6" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="E6">
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="G6" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="H6">
         <v>129320235</v>
@@ -10779,19 +7570,19 @@
         <v>267</v>
       </c>
       <c r="C7" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D7" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="E7">
         <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="G7" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="H7">
         <v>163763691</v>
@@ -10805,22 +7596,22 @@
         <v>250489</v>
       </c>
       <c r="B8" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="C8">
         <v>2007003287</v>
       </c>
       <c r="D8" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="E8">
         <v>40</v>
       </c>
       <c r="F8" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="G8" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="H8">
         <v>779323497</v>
@@ -10837,19 +7628,19 @@
         <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D9" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="E9">
         <v>12</v>
       </c>
       <c r="F9" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="G9" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="H9">
         <v>219344054</v>
@@ -10863,22 +7654,22 @@
         <v>250491</v>
       </c>
       <c r="B10" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="C10" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D10" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="E10">
         <v>26</v>
       </c>
       <c r="F10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="G10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="H10">
         <v>936752533</v>
@@ -10892,22 +7683,22 @@
         <v>250515</v>
       </c>
       <c r="B11" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="C11">
         <v>2013000835</v>
       </c>
       <c r="D11" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="E11">
         <v>11</v>
       </c>
       <c r="F11" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="G11" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="H11">
         <v>1406645617</v>
@@ -10921,22 +7712,22 @@
         <v>250499</v>
       </c>
       <c r="B12" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="C12">
         <v>2007003287</v>
       </c>
       <c r="D12" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="E12">
         <v>44</v>
       </c>
       <c r="F12" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="G12" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="H12">
         <v>1434188792</v>
@@ -10950,22 +7741,22 @@
         <v>250516</v>
       </c>
       <c r="B13" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="C13" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D13" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="E13">
         <v>38</v>
       </c>
       <c r="F13" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="G13" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="H13">
         <v>1689232192</v>
@@ -10979,22 +7770,22 @@
         <v>250517</v>
       </c>
       <c r="B14" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C14" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D14" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="E14">
         <v>24</v>
       </c>
       <c r="F14" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="G14" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="H14">
         <v>331383731</v>
@@ -11011,19 +7802,19 @@
         <v>134</v>
       </c>
       <c r="C15" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D15" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E15">
         <v>25</v>
       </c>
       <c r="F15" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="G15" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="H15">
         <v>587046985</v>
@@ -11037,22 +7828,22 @@
         <v>250493</v>
       </c>
       <c r="B16" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="C16" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D16" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="E16">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="G16" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="H16">
         <v>549545953</v>
@@ -11072,16 +7863,16 @@
         <v>2011000150</v>
       </c>
       <c r="D17" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="E17">
         <v>43</v>
       </c>
       <c r="F17" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="G17" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="H17">
         <v>1034145514</v>
@@ -11095,22 +7886,22 @@
         <v>250495</v>
       </c>
       <c r="B18" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C18" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D18" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="E18">
         <v>16</v>
       </c>
       <c r="F18" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="G18" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="H18">
         <v>729665110</v>
@@ -11124,22 +7915,22 @@
         <v>250496</v>
       </c>
       <c r="B19" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="C19" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D19" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="E19">
         <v>8</v>
       </c>
       <c r="F19" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="G19" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="H19">
         <v>451422310</v>
@@ -11156,19 +7947,19 @@
         <v>160</v>
       </c>
       <c r="C20" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D20" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="E20">
         <v>13</v>
       </c>
       <c r="F20" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="G20" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="H20">
         <v>592749199</v>
@@ -11182,22 +7973,22 @@
         <v>250518</v>
       </c>
       <c r="B21" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="C21" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D21" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="E21">
         <v>27</v>
       </c>
       <c r="F21" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="G21" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="H21">
         <v>126739747</v>
@@ -11217,16 +8008,16 @@
         <v>2016000861</v>
       </c>
       <c r="D22" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="E22">
         <v>7</v>
       </c>
       <c r="F22" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="G22" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="H22">
         <v>965761484</v>
@@ -11240,22 +8031,22 @@
         <v>250500</v>
       </c>
       <c r="B23" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C23" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D23" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="E23">
         <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="G23" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="H23">
         <v>103525518</v>
@@ -11269,22 +8060,22 @@
         <v>250501</v>
       </c>
       <c r="B24" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C24" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D24" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="E24">
         <v>32</v>
       </c>
       <c r="F24" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="G24" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="H24">
         <v>130997296</v>
@@ -11298,22 +8089,22 @@
         <v>250502</v>
       </c>
       <c r="B25" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C25" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D25" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="E25">
         <v>4</v>
       </c>
       <c r="F25" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="G25" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="H25">
         <v>1014359496</v>
@@ -11330,19 +8121,19 @@
         <v>186</v>
       </c>
       <c r="C26" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D26" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="E26">
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="G26" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="H26">
         <v>1006207078</v>
@@ -11356,22 +8147,22 @@
         <v>250505</v>
       </c>
       <c r="B27" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="C27" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D27" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="E27">
         <v>18</v>
       </c>
       <c r="F27" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="G27" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="H27">
         <v>982492835</v>
@@ -11385,22 +8176,22 @@
         <v>250506</v>
       </c>
       <c r="B28" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="C28" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D28" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="E28">
         <v>3</v>
       </c>
       <c r="F28" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="G28" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="H28">
         <v>828299094</v>
@@ -11414,22 +8205,22 @@
         <v>250507</v>
       </c>
       <c r="B29" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="C29">
         <v>2007001374</v>
       </c>
       <c r="D29" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="E29">
         <v>42</v>
       </c>
       <c r="F29" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="G29" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="H29">
         <v>1018448390</v>
@@ -11443,22 +8234,22 @@
         <v>250508</v>
       </c>
       <c r="B30" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="C30" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D30" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="E30">
         <v>17</v>
       </c>
       <c r="F30" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="G30" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="H30">
         <v>69176968</v>
@@ -11475,19 +8266,19 @@
         <v>211</v>
       </c>
       <c r="C31" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D31" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="E31">
         <v>37</v>
       </c>
       <c r="F31" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="G31" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="H31">
         <v>112747114</v>
@@ -11501,22 +8292,22 @@
         <v>250519</v>
       </c>
       <c r="B32" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="C32" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D32" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="E32">
         <v>5</v>
       </c>
       <c r="F32" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="G32" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H32">
         <v>110965961</v>
@@ -11533,19 +8324,19 @@
         <v>223</v>
       </c>
       <c r="C33" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D33" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="E33">
         <v>23</v>
       </c>
       <c r="F33" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="G33" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="H33">
         <v>862464766</v>
@@ -11559,22 +8350,22 @@
         <v>250520</v>
       </c>
       <c r="B34" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C34" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D34" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="E34">
         <v>29</v>
       </c>
       <c r="F34" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="G34" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H34">
         <v>299927960</v>
@@ -11591,19 +8382,19 @@
         <v>237</v>
       </c>
       <c r="C35" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D35" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="E35">
         <v>34</v>
       </c>
       <c r="F35" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="G35" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="H35">
         <v>353933195</v>
@@ -11623,16 +8414,16 @@
         <v>2013000835</v>
       </c>
       <c r="D36" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="E36">
         <v>39</v>
       </c>
       <c r="F36" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="G36" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="H36">
         <v>1324701108</v>
@@ -11646,22 +8437,22 @@
         <v>250521</v>
       </c>
       <c r="B37" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="C37" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D37" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="E37">
         <v>31</v>
       </c>
       <c r="F37" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="G37" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="H37">
         <v>988837201</v>
@@ -11678,19 +8469,19 @@
         <v>255</v>
       </c>
       <c r="C38" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D38" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="E38">
         <v>2</v>
       </c>
       <c r="F38" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="G38" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="H38">
         <v>1005327426</v>
@@ -11704,22 +8495,22 @@
         <v>250514</v>
       </c>
       <c r="B39" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="C39" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D39" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="E39">
         <v>15</v>
       </c>
       <c r="F39" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="G39" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="H39">
         <v>896275816</v>
@@ -11736,16 +8527,16 @@
         <v>0</v>
       </c>
       <c r="D40" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E40" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="F40" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="G40" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="H40">
         <v>254662</v>

</xml_diff>